<commit_message>
fix: Correct caratteristica columns from IDML Family_Tech_Data styles
Applied 50 corrections to caratteristica_primaria, valore_primario,
caratteristica_secondaria, and valore_secondario columns.

Previous values came from wrong IDML section (tech specs table).
Correct values extracted from Family_Tech_Data_gruppo styles:
- Title_Value1 -> caratteristica_primaria
- Family_Tech_Data_Value1 -> valore_primario
- Title_Value2 -> caratteristica_secondaria
- Family_Tech_Data_Value2 -> valore_secondario

Products corrected: 770N 24V, S800H ENC, C4000I, C720, 740, 740 C,
741, 741 C, 746 C, 844 C, 844 3PH, 550, 390 230V, 560
</commit_message>
<xml_diff>
--- a/output/v2/Data_Elena_P_KIT_v4.xlsx
+++ b/output/v2/Data_Elena_P_KIT_v4.xlsx
@@ -5724,22 +5724,22 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Larghezza max singola anta</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2 m (3,5 m con elettroserratura)</t>
+          <t>2 - 3,5 m (con elettroserratura)</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Peso max anta</t>
+          <t>Peso max</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>500 Kg (vedi grafico)</t>
+          <t>500 Kg</t>
         </is>
       </c>
       <c r="O48" t="inlineStr"/>
@@ -5849,22 +5849,22 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Larghezza max singola anta</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>2 m 4 m 2 m 4 m</t>
+          <t>2 - 4 m</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Peso max anta</t>
+          <t>Peso max</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2 - 4 m</t>
+          <t>800 Kg</t>
         </is>
       </c>
       <c r="O49" t="inlineStr"/>
@@ -6100,22 +6100,22 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>8 m</t>
+          <t>400 Kg</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Peso max anta</t>
+          <t>Velocità max</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>400 kg</t>
+          <t>16 m/min</t>
         </is>
       </c>
       <c r="O51" t="inlineStr"/>
@@ -6220,22 +6220,22 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>15 m</t>
+          <t>400 Kg</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Velocità dell'anta</t>
+          <t>Velocità max</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>18 m/min (regolabile)</t>
+          <t>18 m/min.</t>
         </is>
       </c>
       <c r="O52" t="inlineStr"/>
@@ -6466,22 +6466,22 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>15 m</t>
+          <t>500 Kg</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Velocità dell'anta</t>
+          <t>Velocità max</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>12 m/min</t>
+          <t>12 m/min.</t>
         </is>
       </c>
       <c r="O54" t="inlineStr"/>
@@ -6710,22 +6710,22 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>15 m</t>
+          <t>500 Kg</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Peso max anta</t>
+          <t>Velocità max</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>500 Kg</t>
+          <t>12 m/min.</t>
         </is>
       </c>
       <c r="O56" t="n">
@@ -6828,12 +6828,12 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>15 m</t>
+          <t>900 Kg</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>12 m/min</t>
+          <t>12 m/min.</t>
         </is>
       </c>
       <c r="O57" t="inlineStr"/>
@@ -6946,22 +6946,22 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t xml:space="preserve">15 m </t>
+          <t>900 Kg</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Velocità dell'anta</t>
+          <t>Velocità max</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>12 m/min</t>
+          <t>12 m/min.</t>
         </is>
       </c>
       <c r="O58" t="n">
@@ -7063,22 +7063,22 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Potenza max</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>150 W</t>
+          <t>400 - 600 Kg</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Lunghezza max anta</t>
+          <t>Velocità max</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>40 m 50 m</t>
+          <t>9,6 - 12 m/min.</t>
         </is>
       </c>
       <c r="O59" t="inlineStr"/>
@@ -7303,22 +7303,22 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Velocità max anta</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>9.6 m/min</t>
+          <t>1.800 Kg</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Lunghezza max anta</t>
+          <t>Velocità max</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>40 m</t>
+          <t>9,5 - 12 m/min.</t>
         </is>
       </c>
       <c r="O61" t="n">
@@ -7424,22 +7424,22 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Velocità dell'anta</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>9,5 m/min (Z16) - 7,2 m/min (Z12) - 12,0 m/min (Z20)</t>
+          <t>1.600 - 2.200 Kg</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Velocità max</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>30 m (Z12) - 40 m (Z16) - 50 m (Z20)</t>
+          <t>7.2 -9.5- 12 m/min</t>
         </is>
       </c>
       <c r="O62" t="inlineStr"/>
@@ -8105,22 +8105,22 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peso max porta </t>
+          <t>Dimensioni max porta (L X H)</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
+          <t>3 x 2,7 m (4 x 3 m con due attuatori)</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>Peso max porta</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
           <t>10 Kg/mq</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>Peso</t>
-        </is>
-      </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>7,5 Kg</t>
         </is>
       </c>
       <c r="O68" t="inlineStr"/>
@@ -8329,12 +8329,12 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Larghezza max singolo</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>1,8 m (3 m con elettroserratura)</t>
+          <t>1,5 m</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -8442,7 +8442,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Larghezza max singolo pannello</t>
+          <t>Larghezza max singolo</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">

</xml_diff>